<commit_message>
Open Cycle and Hab Updates also v53
</commit_message>
<xml_diff>
--- a/docs/current-implementation-matrix.xlsx
+++ b/docs/current-implementation-matrix.xlsx
@@ -2,7 +2,7 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Implementation Matrix" sheetId="1" r:id="Rc9e35254a22d4887"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Implementation Matrix" sheetId="1" r:id="Rffa6906764564c63"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -2420,28 +2420,28 @@
         <x:v>ships</x:v>
       </x:c>
       <x:c r="C55" s="12" t="str">
-        <x:v>Power-plant output and waste-heat calculation</x:v>
+        <x:v>Open-cycle reactor mass, cap, and compact power presentation</x:v>
       </x:c>
       <x:c r="D55" s="12" t="str">
-        <x:v>Delivered load × (1 - efficiency), which understates input minus output</x:v>
+        <x:v>Open-cycle drive load is presented as reactor electricity; plant mass, cost, output, and heat use one undifferentiated demand.</x:v>
       </x:c>
       <x:c r="E55" s="12" t="str">
         <x:v>No maintained-main override</x:v>
       </x:c>
       <x:c r="F55" s="12" t="str">
-        <x:v>Closed-cycle loads use delivered load × (1 / efficiency - 1). Open-cycle drives require reactor output Q = D / (1 - f × (1 - efficiency)) after hull-art scaling and retain Q - D as ship heat. Plant mass, cost, live generation, compatibility, reactor-bay use, designer display, and combat heat share that demand; powered-weapon module losses remain on the generator-sized burst interval.</x:v>
+        <x:v>Open-cycle drive demand D remains useful thermal GWth; closed-cycle drive and auxiliary demands remain electrical GWe. Gross reactor input is Qoc = D / (1 - f × (1 - efficiency)) plus electrical thermal input. Plant mass, build cost, and reactor-bay occupancy use Pmass = m × Qoc + Qelectrical, while drive cap use is Cdrive = m × Qoc for open cycle and D for closed cycle. Live thermal output and heat retain full energy conservation. As a temporary gameplay calibration pending the reactor rebalance, every reactor class except fuel-cell/general uses a 0.5 open-cycle multiplier; fuel-cell/general plants remain 1.0. The compact UI preserves vanilla Classification, Mass, Crew, Efficiency, Max Output To Drive, and cost rows; replaces installed Output with Electrical Output plus useful Thermal Output D only for open-cycle drives; collapses heat to one Waste Heat row; appends m parenthetically to Specific Power; and keeps reactor-bay volume outside the table.</x:v>
       </x:c>
       <x:c r="G55" s="12" t="str">
-        <x:v>shipBalance.enabled;shipBalance.correctPowerPlantWasteHeat;shipBalance.openCycleResidualHeatEnabled;shipBalance.openCycleDriveHeatFraction</x:v>
+        <x:v>shipBalance.enabled;shipBalance.correctPowerPlantWasteHeat;shipBalance.openCycleResidualHeatEnabled;shipBalance.openCycleDriveHeatFraction;shipBalance.openCycleThermalMassScalingEnabled</x:v>
       </x:c>
       <x:c r="H55" s="12" t="str">
-        <x:v>BalancePatches.cs:PowerPlantWasteHeatPatch;BalancePatches.cs:OpenCycleDrivePowerPlantCompatibilityPatch;BalancePatches.cs:OpenCycleValidDrivesForPowerPlantsPatch;ShipPowerPatches.cs:InstalledDriveHeatPatch;ShipPowerPatches.cs:PoweredWeaponRadiatorHeatPatch;ShipPowerPatches.cs:AuxiliaryElectricalGenerationPatch;ShipPowerPatches.cs:GeneratedPowerHeatPatch;ShipPowerPatches.cs:DuplicateSystemsHeatPatch;ShipPowerPatches.cs:WeaponHeatCapacityPrecheckPatch;Core/PowerPlantThermalMath.cs;Core/WeaponPowerMath.cs;docs/ship-balance-research/open-cycle-reactor-demand-and-heat.md</x:v>
+        <x:v>Core/PowerPlantThermalMath.cs;Core/PowerPlantScalingMath.cs;Core/PowerPlantScalingRegistry.cs;BalancePatches.cs:ShipPowerDemandFeature;BalancePatches.cs:PowerPlantWasteHeatPatch;BalancePatches.cs:SeparatedShipPowerProductionPatch;BalancePatches.cs:OpenCyclePowerPlantMassPatch;BalancePatches.cs:OpenCyclePowerPlantCostPatch;BalancePatches.cs:OpenCycleDrivePowerPlantCompatibilityPatch;BalancePatches.cs:OpenCycleValidDrivesForPowerPlantsPatch;ShipPowerPatches.cs:InstalledDriveHeatPatch;ShipPowerPatches.cs:PoweredWeaponRadiatorHeatPatch;ShipPowerPatches.cs:AuxiliaryElectricalGenerationPatch;ShipPowerPatches.cs:GeneratedPowerHeatPatch;ShipPowerPatches.cs:DuplicateSystemsHeatPatch;ShipPowerPatches.cs:WeaponHeatCapacityPrecheckPatch;TIPowerPlantTemplate.json;UIGeneralControls.en;docs/ship-balance-research/open-cycle-reactor-demand-and-heat.md;docs/ship-balance-research/open-cycle-reactor-mass-scaling-plan-2026-08-21.md</x:v>
       </x:c>
       <x:c r="I55" s="12" t="str">
-        <x:v>updated</x:v>
+        <x:v>implemented</x:v>
       </x:c>
       <x:c r="J55" s="12" t="str">
-        <x:v>Open-cycle reactor demand now conserves useful drive work plus the configured retained loss. Combat burns use the installed ship-level demand, fixing the raw drive-template bypass of hull-art scaling. Candidate and static AI filters enforce the same output boundary. Radiators still cover corrected reactor rejection and explicit weapon-conversion losses exactly once.</x:v>
+        <x:v>All non-fuel-cell/general open-cycle propulsion is temporarily mass- and cap-rated at 50% of gross thermal input so the uneven pre-rebalance reactor progression cannot amplify technology-specific discounts. Authored maxOutput_GW values remain unchanged: 8 GWth open-cycle and 4 GWe closed-cycle each consume 4 GW of rated drive capacity at m = 0.5 before retained-loss correction. Thermal Output in the UI deliberately means useful work D delivered to the open-cycle drive; gross Qoc remains internal.</x:v>
       </x:c>
     </x:row>
     <x:row r="56" ht="39.599998474121094" hidden="0" customHeight="1">
@@ -3930,7 +3930,7 @@
   </x:dataValidations>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R8f1854c3dc04442e"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R52ff3a65611a4e34"/>
   </x:tableParts>
 </x:worksheet>
 </file>
</xml_diff>

<commit_message>
Ship Cache Propellant Cap Fix
</commit_message>
<xml_diff>
--- a/docs/current-implementation-matrix.xlsx
+++ b/docs/current-implementation-matrix.xlsx
@@ -2,7 +2,7 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Implementation Matrix" sheetId="1" r:id="R82d81f10c7434dc4"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Implementation Matrix" sheetId="1" r:id="Re457e96a5cfe432d"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -2781,19 +2781,19 @@
         <x:v>No maintained-main override</x:v>
       </x:c>
       <x:c r="F66" s="11" t="str">
-        <x:v>Gun power is runtime template metadata and adds no save field. On load, ship power statistics use current templates and current mass is reconciled to recalculated dry mass plus saved propellant</x:v>
+        <x:v>Gun power is runtime template metadata and adds no save field. On load, saved faction designs rebuild dry mass, acceleration, delta-v, battery, and heat through the game's aggregate template cache function; instantiated ships use that same refresh before reconciling current mass to recalculated dry mass plus saved propellant.</x:v>
       </x:c>
       <x:c r="G66" s="11" t="str">
         <x:v>shipBalance.enabled</x:v>
       </x:c>
       <x:c r="H66" s="11" t="str">
-        <x:v>GunPowerRegistry.cs;ShipPowerPatches.cs:GunPowerTemplateInitializationPatch;ShipPowerPatches.cs:ShipPowerSaveLoadCachePatch;Main.cs:Main</x:v>
+        <x:v>GunPowerRegistry.cs;ShipPowerPatches.cs:GunPowerTemplateInitializationPatch;ShipPowerPatches.cs:ShipPowerSaveLoadCachePatch;Main.cs:Main;ShipPowerPatches.cs:ShipDesignPerformanceSaveLoadCachePatch</x:v>
       </x:c>
       <x:c r="I66" s="11" t="str">
         <x:v>implemented</x:v>
       </x:c>
       <x:c r="J66" s="11" t="str">
-        <x:v>The registry is rebuilt from active load-ordered mod JSON before a save is selected. TI 1.0.51 late saves retain their saved fuel while propulsion is marked for recalculation, and mixed conventional-gun unlock sets initialize without a module-table exception. Disabling or removing the mod requires no custom save payload.</x:v>
+        <x:v>The registry is rebuilt from active load-ordered mod JSON before a save is selected. TI 1.0.51 late saves retain their saved fuel while propulsion is marked for recalculation, and mixed conventional-gun unlock sets initialize without a module-table exception. Disabling or removing the mod requires no custom save payload. TI 1.0.53 faction designs now refresh every performance cache after save registration, preventing one cached statistic from retaining an older mass model.</x:v>
       </x:c>
     </x:row>
     <x:row r="67" ht="13.5" hidden="0" customHeight="1">
@@ -3421,19 +3421,19 @@
         <x:v>No measured per-art hull-volume fuel cap or hull/engine art-pane readout</x:v>
       </x:c>
       <x:c r="F86" s="12" t="str">
-        <x:v>Measured per-art main-hull volume minus installed utility/weapon footprints and 50 m³ per total fitted crew billet; density-aware 100-ton tanks clamp before designer refresh and save. Human AI designs select an appearance before propulsion sizing, ideal-tank calculations clamp to capacity and recompute achieved delta-v, refits preserve their appearance, and final human/alien/STO save boundaries reject illegal propulsion layouts. The art pane shows selected-art De Laval and Magnetic gameplay scales, Pulsed 1x, measured engine-bay volume, flat empty-hull mass, base repair crew, propellant, tank cap, and usable fuel volume.</x:v>
+        <x:v>Measured per-art main-hull volume minus installed utility/weapon footprints and 50 m³ per total fitted crew billet; density-aware 100-ton tanks clamp during normal designer refresh and save. Existing-template loading preserves the serialized tank count while the UI is assembled, then checks it once against the final saved art and rebuilds cost and performance caches. Human AI designs select an appearance before propulsion sizing, ideal-tank calculations clamp to capacity and recompute achieved delta-v, refits preserve their appearance, and final human/alien/STO save boundaries reject illegal propulsion layouts. The art pane shows selected-art De Laval and Magnetic gameplay scales, Pulsed 1x, measured engine-bay volume, flat empty-hull mass, base repair crew, propellant, tank cap, and usable fuel volume.</x:v>
       </x:c>
       <x:c r="G86" s="12" t="str">
         <x:v>shipBalance.enabled;shipBalance.fuelVolumeCapacityEnabled;shipBalance.utilitySlotVolume_m3;shipBalance.hullWeaponSlotVolume_m3;shipBalance.noseWeaponSlotVolume_m3;shipBalance.crewPressurizedVolume_m3</x:v>
       </x:c>
       <x:c r="H86" s="12" t="str">
-        <x:v>FuelCapacityPatches.cs:PropellantDensityTemplateInitializationPatch;FuelCapacityPatches.cs:FuelCapacityDesignerRefreshPatch;FuelCapacityPatches.cs:FuelCapacitySpinnerLabelPatch;FuelCapacityPatches.cs:FuelCapacitySaveGuardPatch;FuelCapacityPatches.cs:AiShipDesignCapacityBoundaryPatch;FuelCapacityPatches.cs:AiShipRefitCapacityBoundaryPatch;FuelCapacityPatches.cs:AiShipEarlyAppearanceSelectionPatch;FuelCapacityPatches.cs:FuelCapacityIdealTankCountPatch;FuelCapacityPatches.cs:AlienShipFuelCapacityPatch;FuelCapacityPatches.cs:StoFighterFuelCapacityPatch;FuelCapacityPatches.cs:SavedShipCapacityInvariantPatch;Core/HullVolumeCatalog.cs:HullVolumeCatalog;Core/HullDriveScaleCatalog.cs:HullDriveScaleCatalog;Core/PropellantDensityRegistry.cs:PropellantDensityRegistry;Config/hull-variant-main-volumes.csv;Config/hull-variant-drive-scales.csv</x:v>
+        <x:v>FuelCapacityPatches.cs:PropellantDensityTemplateInitializationPatch;FuelCapacityPatches.cs:FuelCapacityDesignerRefreshPatch;FuelCapacityPatches.cs:FuelCapacitySpinnerLabelPatch;FuelCapacityPatches.cs:FuelCapacitySaveGuardPatch;FuelCapacityPatches.cs:AiShipDesignCapacityBoundaryPatch;FuelCapacityPatches.cs:AiShipRefitCapacityBoundaryPatch;FuelCapacityPatches.cs:AiShipEarlyAppearanceSelectionPatch;FuelCapacityPatches.cs:FuelCapacityIdealTankCountPatch;FuelCapacityPatches.cs:AlienShipFuelCapacityPatch;FuelCapacityPatches.cs:StoFighterFuelCapacityPatch;FuelCapacityPatches.cs:SavedShipCapacityInvariantPatch;Core/HullVolumeCatalog.cs:HullVolumeCatalog;Core/HullDriveScaleCatalog.cs:HullDriveScaleCatalog;Core/PropellantDensityRegistry.cs:PropellantDensityRegistry;Config/hull-variant-main-volumes.csv;Config/hull-variant-drive-scales.csv;FuelCapacityPatches.cs:ExistingShipFuelCapacityLoadPatch</x:v>
       </x:c>
       <x:c r="I86" s="12" t="str">
         <x:v>implemented</x:v>
       </x:c>
       <x:c r="J86" s="12" t="str">
-        <x:v>Default footprints are 200 m³ per utility cell, 250 m³ per hull-weapon cell, and 400 m³ per nose-weapon cell. Fuel capacity reserves total fitted crew; the overlay's repair crew is the hull template base complement. De Laval and Magnetic values are the same measured x6 art-envelope ratios consumed by gameplay; Pulsed remains explicitly 1x. Guarded alien and STO transpilers require their exact expected tank-assignment counts and throw rather than allowing a partial patch.</x:v>
+        <x:v>Default footprints are 200 m³ per utility cell, 250 m³ per hull-weapon cell, and 400 m³ per nose-weapon cell. Fuel capacity reserves total fitted crew; the overlay's repair crew is the hull template base complement. De Laval and Magnetic values are the same measured x6 art-envelope ratios consumed by gameplay; Pulsed remains explicitly 1x. Guarded alien and STO transpilers require their exact expected tank-assignment counts and throw rather than allowing a partial patch. The staged Upgrade load no longer lets a lower-capacity intermediate art discard tanks that are legal on the saved appearance.</x:v>
       </x:c>
     </x:row>
     <x:row r="87" ht="150" customHeight="1">
@@ -3962,7 +3962,7 @@
   </x:dataValidations>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R4aadafefd16b4cf0"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R7860713ffeef423b"/>
   </x:tableParts>
 </x:worksheet>
 </file>
</xml_diff>

<commit_message>
Release 0.10.1 with open-cycle fusion drives and heavier human reactors
Set all 174 human and alien fusion-drive variants to explicit Open cooling
and double specificPower_tGW for all 27 human fusion reactors. Use sparse
overrides to preserve other reactor and drive properties, including alien
performance and backup electrical generation settings.

Update the effective reactor and drive tables, implementation matrix, release
metadata, and packaged assembly. Include the fusion research report and
implementation notes explaining the scientific rationale and gameplay scope.
Extend validation to cover every fusion variant and preserve existing values.

Validation: normal deploy.ps1 completed with all 37 validators and 1,204
formula assertions passing; all 47 deployed package files were hash-verified.
Table and workbook checks passed. Manual in-game testing remains pending.
</commit_message>
<xml_diff>
--- a/docs/current-implementation-matrix.xlsx
+++ b/docs/current-implementation-matrix.xlsx
@@ -2,7 +2,7 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Implementation Matrix" sheetId="1" r:id="R64c3fdfbd98a4040"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Implementation Matrix" sheetId="1" r:id="R35cb905a5dfb45ef"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -2441,7 +2441,7 @@
         <x:v>implemented</x:v>
       </x:c>
       <x:c r="J55" s="12" t="str">
-        <x:v>All non-fuel-cell/general open-cycle propulsion is temporarily mass- and cap-rated at 50% of gross thermal input so the uneven pre-rebalance reactor progression cannot amplify technology-specific discounts. Authored maxOutput_GW values remain unchanged: 8 GWth open-cycle and 4 GWe closed-cycle each consume 4 GW of rated drive capacity at m = 0.5 before retained-loss correction. Thermal Output in the UI deliberately means useful work D delivered to the open-cycle drive; gross Qoc remains internal.</x:v>
+        <x:v>Release 0.10.1 doubles specificPower_tGW for all 27 human fusion reactors and explicitly sets Open cooling on all 174 human/alien fusion drive variants. Alien reactor masses remain unchanged. Retains the 0.5 open-cycle thermal mass/cap multiplier and 0.01 residual-loss parameter. Fitted reactor mass need not double because demand also moves to the direct thermal path. Manual designer and saved-ship checks remain pending.</x:v>
       </x:c>
     </x:row>
     <x:row r="56" ht="39.599998474121094" hidden="0" customHeight="1">
@@ -4090,7 +4090,7 @@
   </x:dataValidations>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R3a5e918944f94d58"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R058176c4e10b4c73"/>
   </x:tableParts>
 </x:worksheet>
 </file>
</xml_diff>

<commit_message>
Release 0.10.3 mission probability and alien territory fixes
Floor contested mission chances to 0.1 percentage-point steps, prevent zero-chance orders for players and AI, and use precise rolls with strict success boundaries. Display fractional extremes and exact 0%/100% endpoints.

Promote raw chances strictly above 99.95% to certainty without changing normal critical-success rolls. Retain version 0.10.3 for this adjustment.

Include the previously deployed 0.10.2 full-Servant-control territory-demand restriction so source matches the packaged DLL. Add focused boundary, formatting, assignment, AI, and Harmony validation and release documentation.

Validation: normal build/deploy verification passed, including 1204 formula assertions; deployed DLL hash matches the package. User confirmed the fix landed on 2026-10-01. Leave unrelated save-editing tools and documentation uncommitted.
</commit_message>
<xml_diff>
--- a/docs/current-implementation-matrix.xlsx
+++ b/docs/current-implementation-matrix.xlsx
@@ -2,7 +2,7 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Implementation Matrix" sheetId="1" r:id="R35cb905a5dfb45ef"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Implementation Matrix" sheetId="1" r:id="R447de19d2ecd4dbc"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -13,7 +13,7 @@
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <x:styleSheet xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <x:fonts count="16">
+  <x:fonts count="17">
     <x:font>
       <x:sz val="11"/>
       <x:name val="Carlito"/>
@@ -105,8 +105,13 @@
       <x:color rgb="FF375623"/>
       <x:name val="Carlito"/>
     </x:font>
+    <x:font>
+      <x:sz val="10"/>
+      <x:color rgb="FF000000"/>
+      <x:name val="Arial"/>
+    </x:font>
   </x:fonts>
-  <x:fills count="26">
+  <x:fills count="27">
     <x:fill>
       <x:patternFill patternType="none"/>
     </x:fill>
@@ -233,6 +238,11 @@
         <x:fgColor rgb="FFE2F0D9"/>
       </x:patternFill>
     </x:fill>
+    <x:fill>
+      <x:patternFill patternType="solid">
+        <x:fgColor rgb="FFFFFFFF"/>
+      </x:patternFill>
+    </x:fill>
   </x:fills>
   <x:borders count="1">
     <x:border/>
@@ -240,7 +250,7 @@
   <x:cellStyleXfs count="1">
     <x:xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </x:cellStyleXfs>
-  <x:cellXfs count="72">
+  <x:cellXfs count="76">
     <x:xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <x:xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <x:alignment vertical="top" wrapText="1"/>
@@ -451,6 +461,14 @@
       <x:alignment horizontal="center" vertical="center" wrapText="0"/>
     </x:xf>
     <x:xf numFmtId="0" fontId="15" fillId="4" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="top" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="0" fillId="26" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="16" fillId="26" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="16" fillId="26" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="16" fillId="26" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <x:alignment vertical="top" wrapText="1"/>
     </x:xf>
   </x:cellXfs>
@@ -461,8 +479,8 @@
 </file>
 
 <file path=xl/tables/table1.xml><?xml version="1.0" encoding="utf-8"?>
-<x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="1" name="ImplementationMatrix" displayName="ImplementationMatrix" ref="A1:J106" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
-  <x:autoFilter ref="A1:J106"/>
+<x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="1" name="ImplementationMatrix" displayName="ImplementationMatrix" ref="A1:J107" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
+  <x:autoFilter ref="A1:J107"/>
   <x:tableColumns count="10">
     <x:tableColumn id="1" name="feature_id"/>
     <x:tableColumn id="2" name="category"/>
@@ -4076,6 +4094,38 @@
         <x:v>Other large human appearances round bare hull plus base crew to 100 t. Slot indices and utility footprints preserved; Mothership layout fits the native grid entirely through JSON.</x:v>
       </x:c>
     </x:row>
+    <x:row r="107" ht="150" customHeight="1">
+      <x:c r="A107" s="75" t="str">
+        <x:v>alien_territory_demands</x:v>
+      </x:c>
+      <x:c r="B107" s="75" t="str">
+        <x:v>National politics</x:v>
+      </x:c>
+      <x:c r="C107" s="75" t="str">
+        <x:v>Alien demands require full Servant control</x:v>
+      </x:c>
+      <x:c r="D107" s="75" t="str">
+        <x:v>Native Demand Claim permits a willing executive to surrender a non-capital region.</x:v>
+      </x:c>
+      <x:c r="E107" s="75" t="str">
+        <x:v>No dedicated override.</x:v>
+      </x:c>
+      <x:c r="F107" s="75" t="str">
+        <x:v>0.10.2: Alien demands require Servant ownership of every control point in the target nation. Other factions and human demands retain native eligibility.</x:v>
+      </x:c>
+      <x:c r="G107" s="75" t="str">
+        <x:v>enabled</x:v>
+      </x:c>
+      <x:c r="H107" s="75" t="str">
+        <x:v>Patches/AlienTerritoryDemandPatches.cs:AlienTerritoryDemandTargetsPatch</x:v>
+      </x:c>
+      <x:c r="I107" s="75" t="str">
+        <x:v>implemented</x:v>
+      </x:c>
+      <x:c r="J107" s="75" t="str">
+        <x:v>Mixed or unowned points block new demands. Native claims and other gates remain. Assume Control and already queued demands are unchanged. See docs/alien-territory-demands.md. Manual testing pending.</x:v>
+      </x:c>
+    </x:row>
   </x:sheetData>
   <x:dataValidations count="3">
     <x:dataValidation type="list" sqref="I2:I38">
@@ -4090,7 +4140,7 @@
   </x:dataValidations>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R058176c4e10b4c73"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R19c7c870f91347ff"/>
   </x:tableParts>
 </x:worksheet>
 </file>
</xml_diff>